<commit_message>
Further OFAT and Reform Scenarios
</commit_message>
<xml_diff>
--- a/Thesis/developer_states.xlsx
+++ b/Thesis/developer_states.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rockmtnins-my.sharepoint.com/personal/abigail_weeks_rmi_org/Documents/Documents/GitHub/Thesis/Thesis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="264" documentId="8_{A4B64DE1-C1F9-4DF8-A805-E80C52345F4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F45BABC-6B5F-470E-96B2-DA3D3AFCA013}"/>
+  <xr:revisionPtr revIDLastSave="282" documentId="8_{A4B64DE1-C1F9-4DF8-A805-E80C52345F4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F86A9FB0-9B2C-4488-9B0C-34D92477D784}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{31558D2F-F994-4500-BC80-1C41F5323AB0}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{31558D2F-F994-4500-BC80-1C41F5323AB0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1119,7 +1119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1134,9 +1134,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1483,6 +1480,7 @@
     <col min="3" max="3" width="18.54296875" customWidth="1"/>
     <col min="4" max="4" width="8.7265625" style="5"/>
     <col min="5" max="5" width="12.7265625" customWidth="1"/>
+    <col min="8" max="8" width="11.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
@@ -1519,7 +1517,7 @@
         <f>1/1000</f>
         <v>1E-3</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="2">
         <v>120</v>
       </c>
       <c r="E2" s="2" t="s">
@@ -1543,7 +1541,7 @@
         <f t="shared" ref="C3:C66" si="0">1/1000</f>
         <v>1E-3</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="2">
         <v>109.3</v>
       </c>
       <c r="E3" s="2" t="s">
@@ -1567,7 +1565,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="2">
         <v>440</v>
       </c>
       <c r="E4" s="2" t="s">
@@ -1591,7 +1589,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="2">
         <v>440</v>
       </c>
       <c r="E5" s="2" t="s">
@@ -1615,7 +1613,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="2">
         <v>60</v>
       </c>
       <c r="E6" s="2" t="s">
@@ -1639,7 +1637,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="2">
         <v>40</v>
       </c>
       <c r="E7" s="2" t="s">
@@ -1663,7 +1661,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="2">
         <v>8.4</v>
       </c>
       <c r="E8" s="2" t="s">
@@ -1675,9 +1673,9 @@
       <c r="G8" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="I8" s="5">
-        <f>SUM(D:D)</f>
-        <v>40783.17</v>
+      <c r="I8" s="5" t="e">
+        <f>SUM(#REF!)</f>
+        <v>#REF!</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
@@ -1691,7 +1689,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="2">
         <v>18.149999999999999</v>
       </c>
       <c r="E9" s="2" t="s">
@@ -1715,7 +1713,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="2">
         <v>294.7</v>
       </c>
       <c r="E10" s="2" t="s">
@@ -1739,7 +1737,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="2">
         <v>150</v>
       </c>
       <c r="E11" s="2" t="s">
@@ -1763,7 +1761,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="2">
         <v>30</v>
       </c>
       <c r="E12" s="2" t="s">
@@ -1787,7 +1785,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="2">
         <v>299</v>
       </c>
       <c r="E13" s="2" t="s">
@@ -1811,7 +1809,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="2">
         <v>62.4</v>
       </c>
       <c r="E14" s="2" t="s">
@@ -1835,7 +1833,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="2">
         <v>43.2</v>
       </c>
       <c r="E15" s="2" t="s">
@@ -1859,7 +1857,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="2">
         <v>200</v>
       </c>
       <c r="E16" s="2" t="s">
@@ -1883,7 +1881,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="2">
         <v>500</v>
       </c>
       <c r="E17" s="2" t="s">
@@ -1907,7 +1905,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D18" s="6">
+      <c r="D18" s="2">
         <v>95.1</v>
       </c>
       <c r="E18" s="2" t="s">
@@ -1931,7 +1929,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D19" s="6">
+      <c r="D19" s="2">
         <v>300</v>
       </c>
       <c r="E19" s="2" t="s">
@@ -1955,7 +1953,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D20" s="6">
+      <c r="D20" s="2">
         <v>300</v>
       </c>
       <c r="E20" s="2" t="s">
@@ -1979,7 +1977,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D21" s="6">
+      <c r="D21" s="2">
         <v>118.6</v>
       </c>
       <c r="E21" s="2" t="s">
@@ -2003,7 +2001,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D22" s="6">
+      <c r="D22" s="2">
         <v>200</v>
       </c>
       <c r="E22" s="2" t="s">
@@ -2027,7 +2025,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D23" s="6">
+      <c r="D23" s="2">
         <v>90</v>
       </c>
       <c r="E23" s="2" t="s">
@@ -2051,7 +2049,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D24" s="6">
+      <c r="D24" s="2">
         <v>144</v>
       </c>
       <c r="E24" s="2" t="s">
@@ -2075,7 +2073,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D25" s="6">
+      <c r="D25" s="2">
         <v>100</v>
       </c>
       <c r="E25" s="2" t="s">
@@ -2099,7 +2097,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D26" s="6">
+      <c r="D26" s="2">
         <v>20</v>
       </c>
       <c r="E26" s="2" t="s">
@@ -2123,7 +2121,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D27" s="6">
+      <c r="D27" s="2">
         <v>42.2</v>
       </c>
       <c r="E27" s="2" t="s">
@@ -2147,7 +2145,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D28" s="6">
+      <c r="D28" s="2">
         <v>20</v>
       </c>
       <c r="E28" s="2" t="s">
@@ -2171,7 +2169,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D29" s="6">
+      <c r="D29" s="2">
         <v>150</v>
       </c>
       <c r="E29" s="2" t="s">
@@ -2195,7 +2193,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D30" s="6">
+      <c r="D30" s="2">
         <v>100</v>
       </c>
       <c r="E30" s="2" t="s">
@@ -2219,7 +2217,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D31" s="6">
+      <c r="D31" s="2">
         <v>79.5</v>
       </c>
       <c r="E31" s="2" t="s">
@@ -2243,7 +2241,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D32" s="6">
+      <c r="D32" s="2">
         <v>150</v>
       </c>
       <c r="E32" s="2" t="s">
@@ -2267,7 +2265,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D33" s="6">
+      <c r="D33" s="2">
         <v>150</v>
       </c>
       <c r="E33" s="2" t="s">
@@ -2291,7 +2289,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D34" s="6">
+      <c r="D34" s="2">
         <v>50</v>
       </c>
       <c r="E34" s="2" t="s">
@@ -2315,7 +2313,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D35" s="6">
+      <c r="D35" s="2">
         <v>50</v>
       </c>
       <c r="E35" s="2" t="s">
@@ -2339,7 +2337,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D36" s="6">
+      <c r="D36" s="2">
         <v>300</v>
       </c>
       <c r="E36" s="2" t="s">
@@ -2363,7 +2361,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D37" s="6">
+      <c r="D37" s="2">
         <v>80</v>
       </c>
       <c r="E37" s="2" t="s">
@@ -2387,7 +2385,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D38" s="6">
+      <c r="D38" s="2">
         <v>199</v>
       </c>
       <c r="E38" s="2" t="s">
@@ -2411,7 +2409,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D39" s="6">
+      <c r="D39" s="2">
         <v>100</v>
       </c>
       <c r="E39" s="2" t="s">
@@ -2435,7 +2433,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D40" s="6">
+      <c r="D40" s="2">
         <v>200</v>
       </c>
       <c r="E40" s="2" t="s">
@@ -2459,7 +2457,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D41" s="6">
+      <c r="D41" s="2">
         <v>300</v>
       </c>
       <c r="E41" s="2" t="s">
@@ -2483,7 +2481,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D42" s="6">
+      <c r="D42" s="2">
         <v>200</v>
       </c>
       <c r="E42" s="2" t="s">
@@ -2507,7 +2505,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D43" s="6">
+      <c r="D43" s="2">
         <v>20</v>
       </c>
       <c r="E43" s="2" t="s">
@@ -2531,7 +2529,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D44" s="6">
+      <c r="D44" s="2">
         <v>175</v>
       </c>
       <c r="E44" s="2" t="s">
@@ -2603,7 +2601,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D47" s="6">
+      <c r="D47" s="2">
         <v>200</v>
       </c>
       <c r="E47" s="2" t="s">
@@ -2627,7 +2625,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D48" s="6">
+      <c r="D48" s="2">
         <v>255</v>
       </c>
       <c r="E48" s="2" t="s">
@@ -2651,7 +2649,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D49" s="6">
+      <c r="D49" s="2">
         <v>180</v>
       </c>
       <c r="E49" s="2" t="s">
@@ -2675,7 +2673,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D50" s="6">
+      <c r="D50" s="2">
         <v>52.2</v>
       </c>
       <c r="E50" s="2" t="s">
@@ -2699,7 +2697,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D51" s="6">
+      <c r="D51" s="2">
         <v>100</v>
       </c>
       <c r="E51" s="2" t="s">
@@ -2723,7 +2721,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D52" s="6">
+      <c r="D52" s="2">
         <v>300</v>
       </c>
       <c r="E52" s="2" t="s">
@@ -2747,7 +2745,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D53" s="6">
+      <c r="D53" s="2">
         <v>150</v>
       </c>
       <c r="E53" s="2" t="s">
@@ -2771,7 +2769,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D54" s="6">
+      <c r="D54" s="2">
         <v>150</v>
       </c>
       <c r="E54" s="2" t="s">
@@ -2795,7 +2793,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D55" s="6">
+      <c r="D55" s="2">
         <v>50</v>
       </c>
       <c r="E55" s="2" t="s">
@@ -2819,7 +2817,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D56" s="6">
+      <c r="D56" s="2">
         <v>300</v>
       </c>
       <c r="E56" s="2" t="s">
@@ -2843,7 +2841,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D57" s="6">
+      <c r="D57" s="2">
         <v>300</v>
       </c>
       <c r="E57" s="2" t="s">
@@ -2867,7 +2865,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D58" s="6">
+      <c r="D58" s="2">
         <v>150</v>
       </c>
       <c r="E58" s="2" t="s">
@@ -2891,7 +2889,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D59" s="6">
+      <c r="D59" s="2">
         <v>150</v>
       </c>
       <c r="E59" s="2" t="s">
@@ -2915,7 +2913,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D60" s="6">
+      <c r="D60" s="2">
         <v>100</v>
       </c>
       <c r="E60" s="2" t="s">
@@ -2939,7 +2937,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D61" s="6">
+      <c r="D61" s="2">
         <v>150</v>
       </c>
       <c r="E61" s="2" t="s">
@@ -2963,7 +2961,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D62" s="6">
+      <c r="D62" s="2">
         <v>299.97000000000003</v>
       </c>
       <c r="E62" s="2" t="s">
@@ -2987,7 +2985,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D63" s="6">
+      <c r="D63" s="2">
         <v>260</v>
       </c>
       <c r="E63" s="2" t="s">
@@ -3011,7 +3009,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D64" s="6">
+      <c r="D64" s="2">
         <v>212</v>
       </c>
       <c r="E64" s="2" t="s">
@@ -3035,7 +3033,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D65" s="6">
+      <c r="D65" s="2">
         <v>200</v>
       </c>
       <c r="E65" s="2" t="s">
@@ -3059,7 +3057,7 @@
         <f t="shared" si="0"/>
         <v>1E-3</v>
       </c>
-      <c r="D66" s="6">
+      <c r="D66" s="2">
         <v>255</v>
       </c>
       <c r="E66" s="2" t="s">
@@ -3083,7 +3081,7 @@
         <f t="shared" ref="C67:C130" si="1">1/1000</f>
         <v>1E-3</v>
       </c>
-      <c r="D67" s="6">
+      <c r="D67" s="2">
         <v>190.89</v>
       </c>
       <c r="E67" s="2" t="s">
@@ -3131,7 +3129,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D69" s="6">
+      <c r="D69" s="2">
         <v>300</v>
       </c>
       <c r="E69" s="2" t="s">
@@ -3155,7 +3153,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D70" s="6">
+      <c r="D70" s="2">
         <v>200</v>
       </c>
       <c r="E70" s="2" t="s">
@@ -3179,7 +3177,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D71" s="6">
+      <c r="D71" s="2">
         <v>346</v>
       </c>
       <c r="E71" s="2" t="s">
@@ -3203,7 +3201,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D72" s="6">
+      <c r="D72" s="2">
         <v>100</v>
       </c>
       <c r="E72" s="2" t="s">
@@ -3227,7 +3225,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D73" s="6">
+      <c r="D73" s="2">
         <v>100</v>
       </c>
       <c r="E73" s="2" t="s">
@@ -3251,7 +3249,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D74" s="6">
+      <c r="D74" s="2">
         <v>100</v>
       </c>
       <c r="E74" s="2" t="s">
@@ -3275,7 +3273,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D75" s="6">
+      <c r="D75" s="2">
         <v>150</v>
       </c>
       <c r="E75" s="2" t="s">
@@ -3299,7 +3297,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D76" s="6">
+      <c r="D76" s="2">
         <v>200</v>
       </c>
       <c r="E76" s="2" t="s">
@@ -3323,7 +3321,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D77" s="6">
+      <c r="D77" s="2">
         <v>200</v>
       </c>
       <c r="E77" s="2" t="s">
@@ -3371,7 +3369,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D79" s="6">
+      <c r="D79" s="2">
         <v>100</v>
       </c>
       <c r="E79" s="2" t="s">
@@ -3395,7 +3393,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D80" s="6">
+      <c r="D80" s="2">
         <v>140</v>
       </c>
       <c r="E80" s="2" t="s">
@@ -3419,7 +3417,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D81" s="6">
+      <c r="D81" s="2">
         <v>100</v>
       </c>
       <c r="E81" s="2" t="s">
@@ -3443,7 +3441,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D82" s="6">
+      <c r="D82" s="2">
         <v>210</v>
       </c>
       <c r="E82" s="2" t="s">
@@ -3467,7 +3465,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D83" s="6">
+      <c r="D83" s="2">
         <v>450</v>
       </c>
       <c r="E83" s="2" t="s">
@@ -3491,7 +3489,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D84" s="6">
+      <c r="D84" s="2">
         <v>180</v>
       </c>
       <c r="E84" s="2" t="s">
@@ -3515,7 +3513,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D85" s="6">
+      <c r="D85" s="2">
         <v>55</v>
       </c>
       <c r="E85" s="2" t="s">
@@ -3539,7 +3537,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D86" s="6">
+      <c r="D86" s="2">
         <v>125</v>
       </c>
       <c r="E86" s="2" t="s">
@@ -3563,7 +3561,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D87" s="6">
+      <c r="D87" s="2">
         <v>300</v>
       </c>
       <c r="E87" s="2" t="s">
@@ -3587,7 +3585,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D88" s="6">
+      <c r="D88" s="2">
         <v>140</v>
       </c>
       <c r="E88" s="2" t="s">
@@ -3611,7 +3609,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D89" s="6">
+      <c r="D89" s="2">
         <v>50</v>
       </c>
       <c r="E89" s="2" t="s">
@@ -3635,7 +3633,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D90" s="6">
+      <c r="D90" s="2">
         <v>300</v>
       </c>
       <c r="E90" s="2" t="s">
@@ -3659,7 +3657,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D91" s="6">
+      <c r="D91" s="2">
         <v>800</v>
       </c>
       <c r="E91" s="2" t="s">
@@ -3683,7 +3681,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D92" s="6">
+      <c r="D92" s="2">
         <v>300</v>
       </c>
       <c r="E92" s="2" t="s">
@@ -3707,7 +3705,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D93" s="6">
+      <c r="D93" s="2">
         <v>300</v>
       </c>
       <c r="E93" s="2" t="s">
@@ -3731,7 +3729,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D94" s="6">
+      <c r="D94" s="2">
         <v>300</v>
       </c>
       <c r="E94" s="2" t="s">
@@ -3755,7 +3753,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D95" s="6">
+      <c r="D95" s="2">
         <v>300</v>
       </c>
       <c r="E95" s="2" t="s">
@@ -3779,7 +3777,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D96" s="6">
+      <c r="D96" s="2">
         <v>255</v>
       </c>
       <c r="E96" s="2" t="s">
@@ -3803,7 +3801,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D97" s="6">
+      <c r="D97" s="2">
         <v>54</v>
       </c>
       <c r="E97" s="2" t="s">
@@ -3827,7 +3825,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D98" s="6">
+      <c r="D98" s="2">
         <v>25</v>
       </c>
       <c r="E98" s="2" t="s">
@@ -3851,7 +3849,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D99" s="6">
+      <c r="D99" s="2">
         <v>100</v>
       </c>
       <c r="E99" s="2" t="s">
@@ -3875,7 +3873,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D100" s="6">
+      <c r="D100" s="2">
         <v>500</v>
       </c>
       <c r="E100" s="2" t="s">
@@ -3899,7 +3897,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D101" s="6">
+      <c r="D101" s="2">
         <v>200</v>
       </c>
       <c r="E101" s="2" t="s">
@@ -3923,7 +3921,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D102" s="6">
+      <c r="D102" s="2">
         <v>300</v>
       </c>
       <c r="E102" s="2" t="s">
@@ -3947,7 +3945,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D103" s="6">
+      <c r="D103" s="2">
         <v>50</v>
       </c>
       <c r="E103" s="2" t="s">
@@ -3971,7 +3969,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D104" s="6">
+      <c r="D104" s="2">
         <v>52.2</v>
       </c>
       <c r="E104" s="2" t="s">
@@ -4019,7 +4017,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D106" s="6">
+      <c r="D106" s="2">
         <v>100</v>
       </c>
       <c r="E106" s="2" t="s">
@@ -4043,7 +4041,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D107" s="6">
+      <c r="D107" s="2">
         <v>100</v>
       </c>
       <c r="E107" s="2" t="s">
@@ -4067,7 +4065,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D108" s="6">
+      <c r="D108" s="2">
         <v>35</v>
       </c>
       <c r="E108" s="2" t="s">
@@ -4091,7 +4089,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D109" s="6">
+      <c r="D109" s="2">
         <v>35</v>
       </c>
       <c r="E109" s="2" t="s">
@@ -4115,7 +4113,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D110" s="6">
+      <c r="D110" s="2">
         <v>80</v>
       </c>
       <c r="E110" s="2" t="s">
@@ -4139,7 +4137,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D111" s="6">
+      <c r="D111" s="2">
         <v>75</v>
       </c>
       <c r="E111" s="2" t="s">
@@ -4163,7 +4161,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D112" s="6">
+      <c r="D112" s="2">
         <v>80</v>
       </c>
       <c r="E112" s="2" t="s">
@@ -4187,7 +4185,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D113" s="6">
+      <c r="D113" s="2">
         <v>250</v>
       </c>
       <c r="E113" s="2" t="s">
@@ -4211,7 +4209,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D114" s="6">
+      <c r="D114" s="2">
         <v>126</v>
       </c>
       <c r="E114" s="2" t="s">
@@ -4235,7 +4233,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D115" s="6">
+      <c r="D115" s="2">
         <v>20</v>
       </c>
       <c r="E115" s="2" t="s">
@@ -4259,7 +4257,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D116" s="6">
+      <c r="D116" s="2">
         <v>20</v>
       </c>
       <c r="E116" s="2" t="s">
@@ -4283,7 +4281,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D117" s="6">
+      <c r="D117" s="2">
         <v>126</v>
       </c>
       <c r="E117" s="2" t="s">
@@ -4307,7 +4305,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D118" s="6">
+      <c r="D118" s="2">
         <v>19.989999999999998</v>
       </c>
       <c r="E118" s="2" t="s">
@@ -4331,7 +4329,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D119" s="6">
+      <c r="D119" s="2">
         <v>18</v>
       </c>
       <c r="E119" s="2" t="s">
@@ -4355,7 +4353,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D120" s="6">
+      <c r="D120" s="2">
         <v>23</v>
       </c>
       <c r="E120" s="2" t="s">
@@ -4379,7 +4377,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D121" s="6">
+      <c r="D121" s="2">
         <v>50</v>
       </c>
       <c r="E121" s="2" t="s">
@@ -4403,7 +4401,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D122" s="6">
+      <c r="D122" s="2">
         <v>150</v>
       </c>
       <c r="E122" s="2" t="s">
@@ -4427,7 +4425,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D123" s="6">
+      <c r="D123" s="2">
         <v>70</v>
       </c>
       <c r="E123" s="2" t="s">
@@ -4451,7 +4449,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D124" s="6">
+      <c r="D124" s="2">
         <v>150</v>
       </c>
       <c r="E124" s="2" t="s">
@@ -4475,7 +4473,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D125" s="6">
+      <c r="D125" s="2">
         <v>20</v>
       </c>
       <c r="E125" s="2" t="s">
@@ -4499,7 +4497,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D126" s="6">
+      <c r="D126" s="2">
         <v>240</v>
       </c>
       <c r="E126" s="2" t="s">
@@ -4523,7 +4521,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D127" s="6">
+      <c r="D127" s="2">
         <v>50</v>
       </c>
       <c r="E127" s="2" t="s">
@@ -4547,7 +4545,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D128" s="6">
+      <c r="D128" s="2">
         <v>20</v>
       </c>
       <c r="E128" s="2" t="s">
@@ -4571,7 +4569,7 @@
         <f t="shared" si="1"/>
         <v>1E-3</v>
       </c>
-      <c r="D129" s="6">
+      <c r="D129" s="2">
         <v>140</v>
       </c>
       <c r="E129" s="2" t="s">
@@ -4619,7 +4617,7 @@
         <f t="shared" ref="C131:C194" si="2">1/1000</f>
         <v>1E-3</v>
       </c>
-      <c r="D131" s="6">
+      <c r="D131" s="2">
         <v>65</v>
       </c>
       <c r="E131" s="2" t="s">
@@ -4643,7 +4641,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D132" s="6">
+      <c r="D132" s="2">
         <v>30</v>
       </c>
       <c r="E132" s="2" t="s">
@@ -4667,7 +4665,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D133" s="6">
+      <c r="D133" s="2">
         <v>40</v>
       </c>
       <c r="E133" s="2" t="s">
@@ -4691,7 +4689,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D134" s="6">
+      <c r="D134" s="2">
         <v>50</v>
       </c>
       <c r="E134" s="2" t="s">
@@ -4715,7 +4713,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D135" s="6">
+      <c r="D135" s="2">
         <v>300</v>
       </c>
       <c r="E135" s="2" t="s">
@@ -4739,7 +4737,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D136" s="6">
+      <c r="D136" s="2">
         <v>50</v>
       </c>
       <c r="E136" s="2" t="s">
@@ -4763,7 +4761,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D137" s="6">
+      <c r="D137" s="2">
         <v>98</v>
       </c>
       <c r="E137" s="2" t="s">
@@ -4787,7 +4785,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D138" s="6">
+      <c r="D138" s="2">
         <v>206.6</v>
       </c>
       <c r="E138" s="2" t="s">
@@ -4811,7 +4809,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D139" s="6">
+      <c r="D139" s="2">
         <v>300</v>
       </c>
       <c r="E139" s="2" t="s">
@@ -4835,7 +4833,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D140" s="6">
+      <c r="D140" s="2">
         <v>100</v>
       </c>
       <c r="E140" s="2" t="s">
@@ -4859,7 +4857,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D141" s="6">
+      <c r="D141" s="2">
         <v>148</v>
       </c>
       <c r="E141" s="2" t="s">
@@ -4883,7 +4881,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D142" s="6">
+      <c r="D142" s="2">
         <v>12</v>
       </c>
       <c r="E142" s="2" t="s">
@@ -4907,7 +4905,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D143" s="6">
+      <c r="D143" s="2">
         <v>100</v>
       </c>
       <c r="E143" s="2" t="s">
@@ -4931,7 +4929,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D144" s="6">
+      <c r="D144" s="2">
         <v>15.75</v>
       </c>
       <c r="E144" s="2" t="s">
@@ -4955,7 +4953,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D145" s="6">
+      <c r="D145" s="2">
         <v>75</v>
       </c>
       <c r="E145" s="2" t="s">
@@ -4979,7 +4977,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D146" s="6">
+      <c r="D146" s="2">
         <v>50</v>
       </c>
       <c r="E146" s="2" t="s">
@@ -5003,7 +5001,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D147" s="6">
+      <c r="D147" s="2">
         <v>20</v>
       </c>
       <c r="E147" s="2" t="s">
@@ -5027,7 +5025,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D148" s="6">
+      <c r="D148" s="2">
         <v>20</v>
       </c>
       <c r="E148" s="2" t="s">
@@ -5051,7 +5049,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D149" s="6">
+      <c r="D149" s="2">
         <v>95</v>
       </c>
       <c r="E149" s="2" t="s">
@@ -5075,7 +5073,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D150" s="6">
+      <c r="D150" s="2">
         <v>19.899999999999999</v>
       </c>
       <c r="E150" s="2" t="s">
@@ -5099,7 +5097,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D151" s="6">
+      <c r="D151" s="2">
         <v>20</v>
       </c>
       <c r="E151" s="2" t="s">
@@ -5123,7 +5121,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D152" s="6">
+      <c r="D152" s="2">
         <v>126.5</v>
       </c>
       <c r="E152" s="2" t="s">
@@ -5147,7 +5145,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D153" s="6">
+      <c r="D153" s="2">
         <v>250</v>
       </c>
       <c r="E153" s="2" t="s">
@@ -5171,7 +5169,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D154" s="6">
+      <c r="D154" s="2">
         <v>202.4</v>
       </c>
       <c r="E154" s="2" t="s">
@@ -5195,7 +5193,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D155" s="6">
+      <c r="D155" s="2">
         <v>197.2</v>
       </c>
       <c r="E155" s="2" t="s">
@@ -5219,7 +5217,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D156" s="6">
+      <c r="D156" s="2">
         <v>77</v>
       </c>
       <c r="E156" s="2" t="s">
@@ -5243,7 +5241,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D157" s="6">
+      <c r="D157" s="2">
         <v>150</v>
       </c>
       <c r="E157" s="2" t="s">
@@ -5267,7 +5265,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D158" s="6">
+      <c r="D158" s="2">
         <v>53.9</v>
       </c>
       <c r="E158" s="2" t="s">
@@ -5291,7 +5289,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D159" s="6">
+      <c r="D159" s="2">
         <v>40</v>
       </c>
       <c r="E159" s="2" t="s">
@@ -5315,7 +5313,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D160" s="6">
+      <c r="D160" s="2">
         <v>20</v>
       </c>
       <c r="E160" s="2" t="s">
@@ -5339,7 +5337,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D161" s="6">
+      <c r="D161" s="2">
         <v>20</v>
       </c>
       <c r="E161" s="2" t="s">
@@ -5363,7 +5361,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D162" s="6">
+      <c r="D162" s="2">
         <v>20</v>
       </c>
       <c r="E162" s="2" t="s">
@@ -5387,7 +5385,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D163" s="6">
+      <c r="D163" s="2">
         <v>60</v>
       </c>
       <c r="E163" s="2" t="s">
@@ -5411,7 +5409,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D164" s="6">
+      <c r="D164" s="2">
         <v>100</v>
       </c>
       <c r="E164" s="2" t="s">
@@ -5435,7 +5433,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D165" s="6">
+      <c r="D165" s="2">
         <v>100</v>
       </c>
       <c r="E165" s="2" t="s">
@@ -5459,7 +5457,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D166" s="6">
+      <c r="D166" s="2">
         <v>15</v>
       </c>
       <c r="E166" s="2" t="s">
@@ -5483,7 +5481,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D167" s="6">
+      <c r="D167" s="2">
         <v>15</v>
       </c>
       <c r="E167" s="2" t="s">
@@ -5507,7 +5505,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D168" s="6">
+      <c r="D168" s="2">
         <v>30</v>
       </c>
       <c r="E168" s="2" t="s">
@@ -5531,7 +5529,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D169" s="6">
+      <c r="D169" s="2">
         <v>30</v>
       </c>
       <c r="E169" s="2" t="s">
@@ -5555,7 +5553,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D170" s="6">
+      <c r="D170" s="2">
         <v>174.8</v>
       </c>
       <c r="E170" s="2" t="s">
@@ -5579,7 +5577,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D171" s="6">
+      <c r="D171" s="2">
         <v>50</v>
       </c>
       <c r="E171" s="2" t="s">
@@ -5603,7 +5601,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D172" s="6">
+      <c r="D172" s="2">
         <v>60</v>
       </c>
       <c r="E172" s="2" t="s">
@@ -5627,7 +5625,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D173" s="6">
+      <c r="D173" s="2">
         <v>100</v>
       </c>
       <c r="E173" s="2" t="s">
@@ -5651,7 +5649,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D174" s="6">
+      <c r="D174" s="2">
         <v>80</v>
       </c>
       <c r="E174" s="2" t="s">
@@ -5675,7 +5673,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D175" s="6">
+      <c r="D175" s="2">
         <v>20</v>
       </c>
       <c r="E175" s="2" t="s">
@@ -5699,7 +5697,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D176" s="6">
+      <c r="D176" s="2">
         <v>55</v>
       </c>
       <c r="E176" s="2" t="s">
@@ -5723,7 +5721,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D177" s="6">
+      <c r="D177" s="2">
         <v>20</v>
       </c>
       <c r="E177" s="2" t="s">
@@ -5747,7 +5745,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D178" s="6">
+      <c r="D178" s="2">
         <v>20</v>
       </c>
       <c r="E178" s="2" t="s">
@@ -5771,7 +5769,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D179" s="6">
+      <c r="D179" s="2">
         <v>41</v>
       </c>
       <c r="E179" s="2" t="s">
@@ -5795,7 +5793,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D180" s="6">
+      <c r="D180" s="2">
         <v>25</v>
       </c>
       <c r="E180" s="2" t="s">
@@ -5819,7 +5817,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D181" s="6">
+      <c r="D181" s="2">
         <v>65</v>
       </c>
       <c r="E181" s="2" t="s">
@@ -5843,7 +5841,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D182" s="6">
+      <c r="D182" s="2">
         <v>50</v>
       </c>
       <c r="E182" s="2" t="s">
@@ -5867,7 +5865,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D183" s="6">
+      <c r="D183" s="2">
         <v>75</v>
       </c>
       <c r="E183" s="2" t="s">
@@ -5891,7 +5889,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D184" s="6">
+      <c r="D184" s="2">
         <v>150</v>
       </c>
       <c r="E184" s="2" t="s">
@@ -5915,7 +5913,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D185" s="6">
+      <c r="D185" s="2">
         <v>150</v>
       </c>
       <c r="E185" s="2" t="s">
@@ -5939,7 +5937,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D186" s="6">
+      <c r="D186" s="2">
         <v>200</v>
       </c>
       <c r="E186" s="2" t="s">
@@ -5963,7 +5961,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D187" s="6">
+      <c r="D187" s="2">
         <v>50</v>
       </c>
       <c r="E187" s="2" t="s">
@@ -5987,7 +5985,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D188" s="6">
+      <c r="D188" s="2">
         <v>46.8</v>
       </c>
       <c r="E188" s="2" t="s">
@@ -6011,7 +6009,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D189" s="6">
+      <c r="D189" s="2">
         <v>150</v>
       </c>
       <c r="E189" s="2" t="s">
@@ -6035,7 +6033,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D190" s="6">
+      <c r="D190" s="2">
         <v>150</v>
       </c>
       <c r="E190" s="2" t="s">
@@ -6059,7 +6057,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D191" s="6">
+      <c r="D191" s="2">
         <v>75</v>
       </c>
       <c r="E191" s="2" t="s">
@@ -6083,7 +6081,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D192" s="6">
+      <c r="D192" s="2">
         <v>20</v>
       </c>
       <c r="E192" s="2" t="s">
@@ -6107,7 +6105,7 @@
         <f t="shared" si="2"/>
         <v>1E-3</v>
       </c>
-      <c r="D193" s="6">
+      <c r="D193" s="2">
         <v>200</v>
       </c>
       <c r="E193" s="2" t="s">
@@ -6179,7 +6177,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D196" s="6">
+      <c r="D196" s="2">
         <v>127</v>
       </c>
       <c r="E196" s="2" t="s">
@@ -6203,7 +6201,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D197" s="6">
+      <c r="D197" s="2">
         <v>53</v>
       </c>
       <c r="E197" s="2" t="s">
@@ -6227,7 +6225,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D198" s="6">
+      <c r="D198" s="2">
         <v>60</v>
       </c>
       <c r="E198" s="2" t="s">
@@ -6251,7 +6249,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D199" s="6">
+      <c r="D199" s="2">
         <v>569</v>
       </c>
       <c r="E199" s="2" t="s">
@@ -6275,7 +6273,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D200" s="6">
+      <c r="D200" s="2">
         <v>75</v>
       </c>
       <c r="E200" s="2" t="s">
@@ -6299,7 +6297,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D201" s="6">
+      <c r="D201" s="2">
         <v>122</v>
       </c>
       <c r="E201" s="2" t="s">
@@ -6323,7 +6321,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D202" s="6">
+      <c r="D202" s="2">
         <v>314</v>
       </c>
       <c r="E202" s="2" t="s">
@@ -6347,7 +6345,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D203" s="6">
+      <c r="D203" s="2">
         <v>74.5</v>
       </c>
       <c r="E203" s="2" t="s">
@@ -6371,7 +6369,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D204" s="6">
+      <c r="D204" s="2">
         <v>20</v>
       </c>
       <c r="E204" s="2" t="s">
@@ -6395,7 +6393,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D205" s="6">
+      <c r="D205" s="2">
         <v>70</v>
       </c>
       <c r="E205" s="2" t="s">
@@ -6419,7 +6417,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D206" s="6">
+      <c r="D206" s="2">
         <v>127.86</v>
       </c>
       <c r="E206" s="2" t="s">
@@ -6443,7 +6441,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D207" s="6">
+      <c r="D207" s="2">
         <v>130</v>
       </c>
       <c r="E207" s="2" t="s">
@@ -6491,7 +6489,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D209" s="6">
+      <c r="D209" s="2">
         <v>150</v>
       </c>
       <c r="E209" s="2" t="s">
@@ -6515,7 +6513,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D210" s="6">
+      <c r="D210" s="2">
         <v>82.5</v>
       </c>
       <c r="E210" s="2" t="s">
@@ -6539,7 +6537,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D211" s="6">
+      <c r="D211" s="2">
         <v>18</v>
       </c>
       <c r="E211" s="2" t="s">
@@ -6563,7 +6561,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D212" s="6">
+      <c r="D212" s="2">
         <v>75</v>
       </c>
       <c r="E212" s="2" t="s">
@@ -6587,7 +6585,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D213" s="6">
+      <c r="D213" s="2">
         <v>150</v>
       </c>
       <c r="E213" s="2" t="s">
@@ -6611,7 +6609,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D214" s="6">
+      <c r="D214" s="2">
         <v>90</v>
       </c>
       <c r="E214" s="2" t="s">
@@ -6635,7 +6633,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D215" s="6">
+      <c r="D215" s="2">
         <v>36</v>
       </c>
       <c r="E215" s="2" t="s">
@@ -6659,7 +6657,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D216" s="6">
+      <c r="D216" s="2">
         <v>80</v>
       </c>
       <c r="E216" s="2" t="s">
@@ -6683,7 +6681,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D217" s="6">
+      <c r="D217" s="2">
         <v>500</v>
       </c>
       <c r="E217" s="2" t="s">
@@ -6707,7 +6705,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D218" s="6">
+      <c r="D218" s="2">
         <v>72</v>
       </c>
       <c r="E218" s="2" t="s">
@@ -6731,7 +6729,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D219" s="6">
+      <c r="D219" s="2">
         <v>54</v>
       </c>
       <c r="E219" s="2" t="s">
@@ -6755,7 +6753,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D220" s="6">
+      <c r="D220" s="2">
         <v>100</v>
       </c>
       <c r="E220" s="2" t="s">
@@ -6779,7 +6777,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D221" s="6">
+      <c r="D221" s="2">
         <v>100</v>
       </c>
       <c r="E221" s="2" t="s">
@@ -6803,7 +6801,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D222" s="6">
+      <c r="D222" s="2">
         <v>30</v>
       </c>
       <c r="E222" s="2" t="s">
@@ -6827,7 +6825,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D223" s="6">
+      <c r="D223" s="2">
         <v>70</v>
       </c>
       <c r="E223" s="2" t="s">
@@ -6851,7 +6849,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D224" s="6">
+      <c r="D224" s="2">
         <v>63</v>
       </c>
       <c r="E224" s="2" t="s">
@@ -6875,7 +6873,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D225" s="6">
+      <c r="D225" s="2">
         <v>94</v>
       </c>
       <c r="E225" s="2" t="s">
@@ -6899,7 +6897,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D226" s="6">
+      <c r="D226" s="2">
         <v>150</v>
       </c>
       <c r="E226" s="2" t="s">
@@ -6923,7 +6921,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D227" s="6">
+      <c r="D227" s="2">
         <v>117</v>
       </c>
       <c r="E227" s="2" t="s">
@@ -6947,7 +6945,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D228" s="6">
+      <c r="D228" s="2">
         <v>20</v>
       </c>
       <c r="E228" s="2" t="s">
@@ -6971,7 +6969,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D229" s="6">
+      <c r="D229" s="2">
         <v>90</v>
       </c>
       <c r="E229" s="2" t="s">
@@ -6995,7 +6993,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D230" s="6">
+      <c r="D230" s="2">
         <v>107</v>
       </c>
       <c r="E230" s="2" t="s">
@@ -7019,7 +7017,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D231" s="6">
+      <c r="D231" s="2">
         <v>118.56</v>
       </c>
       <c r="E231" s="2" t="s">
@@ -7043,7 +7041,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D232" s="6">
+      <c r="D232" s="2">
         <v>75</v>
       </c>
       <c r="E232" s="2" t="s">
@@ -7067,7 +7065,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D233" s="6">
+      <c r="D233" s="2">
         <v>75</v>
       </c>
       <c r="E233" s="2" t="s">
@@ -7091,7 +7089,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D234" s="6">
+      <c r="D234" s="2">
         <v>26</v>
       </c>
       <c r="E234" s="2" t="s">
@@ -7115,7 +7113,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D235" s="6">
+      <c r="D235" s="2">
         <v>26</v>
       </c>
       <c r="E235" s="2" t="s">
@@ -7139,7 +7137,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D236" s="6">
+      <c r="D236" s="2">
         <v>90</v>
       </c>
       <c r="E236" s="2" t="s">
@@ -7163,7 +7161,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D237" s="6">
+      <c r="D237" s="2">
         <v>150</v>
       </c>
       <c r="E237" s="2" t="s">
@@ -7187,7 +7185,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D238" s="6">
+      <c r="D238" s="2">
         <v>20</v>
       </c>
       <c r="E238" s="2" t="s">
@@ -7211,7 +7209,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D239" s="6">
+      <c r="D239" s="2">
         <v>15</v>
       </c>
       <c r="E239" s="2" t="s">
@@ -7235,7 +7233,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D240" s="6">
+      <c r="D240" s="2">
         <v>15</v>
       </c>
       <c r="E240" s="2" t="s">
@@ -7259,7 +7257,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D241" s="6">
+      <c r="D241" s="2">
         <v>15</v>
       </c>
       <c r="E241" s="2" t="s">
@@ -7283,7 +7281,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D242" s="6">
+      <c r="D242" s="2">
         <v>10</v>
       </c>
       <c r="E242" s="2" t="s">
@@ -7307,7 +7305,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D243" s="6">
+      <c r="D243" s="2">
         <v>150</v>
       </c>
       <c r="E243" s="2" t="s">
@@ -7355,7 +7353,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D245" s="6">
+      <c r="D245" s="2">
         <v>80</v>
       </c>
       <c r="E245" s="2" t="s">
@@ -7379,7 +7377,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D246" s="6">
+      <c r="D246" s="2">
         <v>20</v>
       </c>
       <c r="E246" s="2" t="s">
@@ -7403,7 +7401,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D247" s="6">
+      <c r="D247" s="2">
         <v>60</v>
       </c>
       <c r="E247" s="2" t="s">
@@ -7427,7 +7425,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D248" s="6">
+      <c r="D248" s="2">
         <v>102</v>
       </c>
       <c r="E248" s="2" t="s">
@@ -7451,7 +7449,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D249" s="6">
+      <c r="D249" s="2">
         <v>75</v>
       </c>
       <c r="E249" s="2" t="s">
@@ -7475,7 +7473,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D250" s="6">
+      <c r="D250" s="2">
         <v>50</v>
       </c>
       <c r="E250" s="2" t="s">
@@ -7499,7 +7497,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D251" s="6">
+      <c r="D251" s="2">
         <v>150</v>
       </c>
       <c r="E251" s="2" t="s">
@@ -7523,7 +7521,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D252" s="6">
+      <c r="D252" s="2">
         <v>75</v>
       </c>
       <c r="E252" s="2" t="s">
@@ -7547,7 +7545,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D253" s="6">
+      <c r="D253" s="2">
         <v>62</v>
       </c>
       <c r="E253" s="2" t="s">
@@ -7571,7 +7569,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D254" s="6">
+      <c r="D254" s="2">
         <v>60</v>
       </c>
       <c r="E254" s="2" t="s">
@@ -7595,7 +7593,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D255" s="6">
+      <c r="D255" s="2">
         <v>100</v>
       </c>
       <c r="E255" s="2" t="s">
@@ -7619,7 +7617,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D256" s="6">
+      <c r="D256" s="2">
         <v>100</v>
       </c>
       <c r="E256" s="2" t="s">
@@ -7643,7 +7641,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D257" s="6">
+      <c r="D257" s="2">
         <v>20</v>
       </c>
       <c r="E257" s="2" t="s">
@@ -7667,7 +7665,7 @@
         <f t="shared" si="3"/>
         <v>1E-3</v>
       </c>
-      <c r="D258" s="6">
+      <c r="D258" s="2">
         <v>62.5</v>
       </c>
       <c r="E258" s="2" t="s">
@@ -7691,7 +7689,7 @@
         <f t="shared" ref="C259:C312" si="4">1/1000</f>
         <v>1E-3</v>
       </c>
-      <c r="D259" s="6">
+      <c r="D259" s="2">
         <v>14.2</v>
       </c>
       <c r="E259" s="2" t="s">
@@ -7715,7 +7713,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D260" s="6">
+      <c r="D260" s="2">
         <v>128</v>
       </c>
       <c r="E260" s="2" t="s">
@@ -7739,7 +7737,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D261" s="6">
+      <c r="D261" s="2">
         <v>160</v>
       </c>
       <c r="E261" s="2" t="s">
@@ -7763,7 +7761,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D262" s="6">
+      <c r="D262" s="2">
         <v>20</v>
       </c>
       <c r="E262" s="2" t="s">
@@ -7787,7 +7785,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D263" s="6">
+      <c r="D263" s="2">
         <v>150</v>
       </c>
       <c r="E263" s="2" t="s">
@@ -7811,7 +7809,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D264" s="6">
+      <c r="D264" s="2">
         <v>150</v>
       </c>
       <c r="E264" s="2" t="s">
@@ -7835,7 +7833,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D265" s="6">
+      <c r="D265" s="2">
         <v>500</v>
       </c>
       <c r="E265" s="2" t="s">
@@ -7859,7 +7857,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D266" s="6">
+      <c r="D266" s="2">
         <v>50</v>
       </c>
       <c r="E266" s="2" t="s">
@@ -7931,7 +7929,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D269" s="6">
+      <c r="D269" s="2">
         <v>127.5</v>
       </c>
       <c r="E269" s="2" t="s">
@@ -7955,7 +7953,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D270" s="6">
+      <c r="D270" s="2">
         <v>100</v>
       </c>
       <c r="E270" s="2" t="s">
@@ -7979,7 +7977,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D271" s="6">
+      <c r="D271" s="2">
         <v>100</v>
       </c>
       <c r="E271" s="2" t="s">
@@ -8003,7 +8001,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D272" s="6">
+      <c r="D272" s="2">
         <v>833</v>
       </c>
       <c r="E272" s="2" t="s">
@@ -8027,7 +8025,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D273" s="6">
+      <c r="D273" s="2">
         <v>836</v>
       </c>
       <c r="E273" s="2" t="s">
@@ -8051,7 +8049,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D274" s="6">
+      <c r="D274" s="2">
         <v>820</v>
       </c>
       <c r="E274" s="2" t="s">
@@ -8075,7 +8073,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D275" s="6">
+      <c r="D275" s="2">
         <v>800.1</v>
       </c>
       <c r="E275" s="2" t="s">
@@ -8099,7 +8097,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D276" s="6">
+      <c r="D276" s="2">
         <v>800.1</v>
       </c>
       <c r="E276" s="2" t="s">
@@ -8123,7 +8121,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D277" s="6">
+      <c r="D277" s="2">
         <v>75</v>
       </c>
       <c r="E277" s="2" t="s">
@@ -8147,7 +8145,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D278" s="6">
+      <c r="D278" s="2">
         <v>79</v>
       </c>
       <c r="E278" s="2" t="s">
@@ -8175,7 +8173,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D279" s="6">
+      <c r="D279" s="2">
         <v>260</v>
       </c>
       <c r="E279" s="2" t="s">
@@ -8186,6 +8184,10 @@
       </c>
       <c r="G279" s="2" t="s">
         <v>336</v>
+      </c>
+      <c r="H279">
+        <f>100-(3000/H278)</f>
+        <v>99.926440244836286</v>
       </c>
     </row>
     <row r="280" spans="1:8" x14ac:dyDescent="0.35">
@@ -8199,7 +8201,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D280" s="6">
+      <c r="D280" s="2">
         <v>90</v>
       </c>
       <c r="E280" s="2" t="s">
@@ -8223,7 +8225,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D281" s="6">
+      <c r="D281" s="2">
         <v>250</v>
       </c>
       <c r="E281" s="2" t="s">
@@ -8247,7 +8249,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D282" s="6">
+      <c r="D282" s="2">
         <v>167</v>
       </c>
       <c r="E282" s="2" t="s">
@@ -8258,6 +8260,10 @@
       </c>
       <c r="G282" s="2" t="s">
         <v>336</v>
+      </c>
+      <c r="H282" s="5">
+        <f>(3/41)</f>
+        <v>7.3170731707317069E-2</v>
       </c>
     </row>
     <row r="283" spans="1:8" x14ac:dyDescent="0.35">
@@ -8271,7 +8277,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D283" s="6">
+      <c r="D283" s="2">
         <v>20</v>
       </c>
       <c r="E283" s="2" t="s">
@@ -8295,7 +8301,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D284" s="6">
+      <c r="D284" s="2">
         <v>20</v>
       </c>
       <c r="E284" s="2" t="s">
@@ -8319,7 +8325,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D285" s="6">
+      <c r="D285" s="2">
         <v>20</v>
       </c>
       <c r="E285" s="2" t="s">
@@ -8343,7 +8349,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D286" s="6">
+      <c r="D286" s="2">
         <v>125</v>
       </c>
       <c r="E286" s="2" t="s">
@@ -8391,7 +8397,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D288" s="6">
+      <c r="D288" s="2">
         <v>150</v>
       </c>
       <c r="E288" s="2" t="s">
@@ -8415,7 +8421,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D289" s="6">
+      <c r="D289" s="2">
         <v>20</v>
       </c>
       <c r="E289" s="2" t="s">
@@ -8439,7 +8445,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D290" s="6">
+      <c r="D290" s="2">
         <v>80</v>
       </c>
       <c r="E290" s="2" t="s">
@@ -8463,7 +8469,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D291" s="6">
+      <c r="D291" s="2">
         <v>188.5</v>
       </c>
       <c r="E291" s="2" t="s">
@@ -8487,7 +8493,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D292" s="6">
+      <c r="D292" s="2">
         <v>45</v>
       </c>
       <c r="E292" s="2" t="s">
@@ -8511,7 +8517,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D293" s="6">
+      <c r="D293" s="2">
         <v>55</v>
       </c>
       <c r="E293" s="2" t="s">
@@ -8535,7 +8541,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D294" s="6">
+      <c r="D294" s="2">
         <v>50</v>
       </c>
       <c r="E294" s="2" t="s">
@@ -8559,7 +8565,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D295" s="6">
+      <c r="D295" s="2">
         <v>200</v>
       </c>
       <c r="E295" s="2" t="s">
@@ -8583,7 +8589,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D296" s="6">
+      <c r="D296" s="2">
         <v>106</v>
       </c>
       <c r="E296" s="2" t="s">
@@ -8607,7 +8613,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D297" s="6">
+      <c r="D297" s="2">
         <v>65</v>
       </c>
       <c r="E297" s="2" t="s">
@@ -8631,7 +8637,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D298" s="6">
+      <c r="D298" s="2">
         <v>90</v>
       </c>
       <c r="E298" s="2" t="s">
@@ -8655,7 +8661,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D299" s="6">
+      <c r="D299" s="2">
         <v>100</v>
       </c>
       <c r="E299" s="2" t="s">
@@ -8679,7 +8685,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D300" s="6">
+      <c r="D300" s="2">
         <v>250</v>
       </c>
       <c r="E300" s="2" t="s">
@@ -8703,7 +8709,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D301" s="6">
+      <c r="D301" s="2">
         <v>225</v>
       </c>
       <c r="E301" s="2" t="s">
@@ -8727,7 +8733,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D302" s="6">
+      <c r="D302" s="2">
         <v>222</v>
       </c>
       <c r="E302" s="2" t="s">
@@ -8751,7 +8757,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D303" s="6">
+      <c r="D303" s="2">
         <v>150</v>
       </c>
       <c r="E303" s="2" t="s">
@@ -8775,7 +8781,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D304" s="6">
+      <c r="D304" s="2">
         <v>50</v>
       </c>
       <c r="E304" s="2" t="s">
@@ -8799,7 +8805,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D305" s="6">
+      <c r="D305" s="2">
         <v>120</v>
       </c>
       <c r="E305" s="2" t="s">
@@ -8823,7 +8829,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D306" s="6">
+      <c r="D306" s="2">
         <v>82</v>
       </c>
       <c r="E306" s="2" t="s">
@@ -8847,7 +8853,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D307" s="6">
+      <c r="D307" s="2">
         <v>70</v>
       </c>
       <c r="E307" s="2" t="s">
@@ -8871,7 +8877,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D308" s="6">
+      <c r="D308" s="2">
         <v>57</v>
       </c>
       <c r="E308" s="2" t="s">
@@ -8895,7 +8901,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D309" s="6">
+      <c r="D309" s="2">
         <v>22</v>
       </c>
       <c r="E309" s="2" t="s">
@@ -8919,7 +8925,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D310" s="6">
+      <c r="D310" s="2">
         <v>98</v>
       </c>
       <c r="E310" s="2" t="s">
@@ -8943,7 +8949,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D311" s="6">
+      <c r="D311" s="2">
         <v>64.2</v>
       </c>
       <c r="E311" s="2" t="s">
@@ -8967,7 +8973,7 @@
         <f t="shared" si="4"/>
         <v>1E-3</v>
       </c>
-      <c r="D312" s="6">
+      <c r="D312" s="2">
         <v>120</v>
       </c>
       <c r="E312" s="2" t="s">

</xml_diff>